<commit_message>
feat: update environment variable loading and expand job filtering criteria to include medium priority jobs
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6200" activeTab="1"/>
+    <workbookView windowWidth="19200" windowHeight="6800" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="All Jobs" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="53">
   <si>
     <t>title</t>
   </si>
@@ -70,97 +70,148 @@
     <t>notes</t>
   </si>
   <si>
-    <t>Data Analyst – SQL/Power BI</t>
-  </si>
-  <si>
-    <t>Innover Digital</t>
-  </si>
-  <si>
-    <t>LinkedIn</t>
-  </si>
-  <si>
-    <t>MEDIUM</t>
+    <t>Data Analyst</t>
+  </si>
+  <si>
+    <t>Virtuoso Staffing Solutions</t>
+  </si>
+  <si>
+    <t>Naukri</t>
+  </si>
+  <si>
+    <t>🔥 HIGH</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>https://in.linkedin.com/jobs/view/data-analyst-%E2%80%93-sql-power-bi-at-innover-digital-4395942366?position=10&amp;pageNum=0&amp;refId=tI%2FAq8zu1%2BQJFxa8XMqtSQ%3D%3D&amp;trackingId=93%2F1Mt0lIY%2Fzc4SEkyG56A%3D%3D</t>
-  </si>
-  <si>
-    <t>Results-driven Data Analyst with 3+ years of experience using SQL, Python, and Power BI to extract insights from data and improve business decisions. Proven ability to write complex SQL queries, analyze trends, and automate reporting to support data-driven strategies. Strong foundation in data visualization, statistical analysis, and cloud platforms like Azure.</t>
+    <t>https://www.naukri.com/job-listings-data-analyst-virtuoso-staffing-solutions-bengaluru-2-to-6-years-241225022830</t>
+  </si>
+  <si>
+    <t>Results-driven Data Analyst with 3+ years of experience using Python, SQL, and data visualization tools to uncover insights and improve decision-making. Built interactive reports and dashboards by analyzing data with Pandas, MySQL, and PostgreSQL to support business needs. Strong foundation in Azure and hands-on experience automating workflows and detecting patterns through clean, efficient code.</t>
+  </si>
+  <si>
+    <t>Hi there,
+I came across the Data Analyst role at Virtuoso Staffing Solutions and it really caught my eye. The focus on analytics and data-driven decision making aligns perfectly with what I love doing and what I’ve been working on at Cognizant.
+At Cognizant, I’ve spent the last few years using Python, SQL, and tools like Pandas and NumPy to analyze data, build reports, and uncover insights—whether it was spotting patterns in website data or debugging issues using system metrics. I’ve also worked with MySQL and PostgreSQL to write queries for reporting and validation, and I’ve built small projects like a customer churn prediction model and automated reporting systems. While I haven’t used Tableau or Power BI yet, I’m eager to learn and apply my existing skills in this role.
+I’d love the chance to bring my experience to your team and contribute right away. Looking forward to hearing from you!</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>Applied</t>
+  </si>
+  <si>
+    <t>2026-05-06</t>
+  </si>
+  <si>
+    <t>Gokaldas Exports</t>
+  </si>
+  <si>
+    <t>https://www.naukri.com/job-listings-data-analyst-gokaldas-exports-ltd-bangalore-bengaluru-2-to-4-years-080426933843</t>
+  </si>
+  <si>
+    <t>Detail-oriented Data Analyst with 3+ years of experience using SQL, Python, and analytics tools to uncover insights from data. Skilled in writing SQL queries, creating reports, and identifying patterns to support data-driven decisions. Strong foundation in data analysis, visualization, and problem-solving for business needs.</t>
   </si>
   <si>
     <t>Dear Hiring Team,
-I’m excited about the Data Analyst role at Innover Digital because I admire how the company leverages data to drive meaningful insights for clients. With my background in SQL, Python, and analytics, I’m eager to contribute to a team that values both technical skills and real-world impact.
-At Cognizant, I’ve spent the last three years analyzing data with SQL and Python to uncover patterns, validate reports, and troubleshoot issues—just like what this role requires. My work on projects like customer churn prediction and operations analytics has sharpened my ability to turn raw data into clear, actionable insights. I’m comfortable with MySQL, PostgreSQL, and tools like Pandas, which I know are key for this position.
-I’d love the chance to bring this experience to Innover Digital. Looking forward to discussing how I can help your team.</t>
-  </si>
-  <si>
-    <t>yes</t>
-  </si>
-  <si>
-    <t>Ready to Apply</t>
-  </si>
-  <si>
-    <t>2026-05-05</t>
-  </si>
-  <si>
-    <t>Data Analyst (SQL,HDFS, Hive)</t>
-  </si>
-  <si>
-    <t>RiskInsight Consulting Pvt Ltd.</t>
-  </si>
-  <si>
-    <t>https://in.linkedin.com/jobs/view/data-analyst-sql-hdfs-hive-at-riskinsight-consulting-pvt-ltd-4370337080?position=7&amp;pageNum=0&amp;refId=tI%2FAq8zu1%2BQJFxa8XMqtSQ%3D%3D&amp;trackingId=C62gomGv6bWUIhfZ87iqsA%3D%3D</t>
-  </si>
-  <si>
-    <t>Data Analyst with 3+ years of experience using SQL, Python, and data pipelines to extract insights from large datasets. Skilled in querying databases (MySQL, PostgreSQL), analyzing trends, and automating reports—with hands-on work in HDFS environments. Strong foundation in analytics tools (Pandas, NumPy, Jupyter) and cloud basics (Azure AZ-900) to drive data-driven decisions.</t>
-  </si>
-  <si>
-    <t>Error: Connection error.</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Error</t>
-  </si>
-  <si>
-    <t>Data Analyst - Google Sheets, SQL, Linux/Unix</t>
-  </si>
-  <si>
-    <t>Qualitest</t>
-  </si>
-  <si>
-    <t>https://in.linkedin.com/jobs/view/data-analyst-google-sheets-sql-linux-unix-at-qualitest-4395947428?position=34&amp;pageNum=0&amp;refId=tI%2FAq8zu1%2BQJFxa8XMqtSQ%3D%3D&amp;trackingId=6K7lL%2Feua7x2LrnSRtzTtw%3D%3D</t>
-  </si>
-  <si>
-    <t>Data Analyst with 3+ years of experience using SQL, Python, and Excel to analyze data, build reports, and solve problems. Strong in Google Sheets, SQL queries, and Linux/Unix basics for data tasks. Proven track record of turning raw data into clear insights for teams and projects.</t>
+I’m excited to apply for the Data Analyst role at Gokaldas Exports. As someone who enjoys turning data into actionable insights, I’d love to contribute to a company known for its impact in the textile industry, especially with my background in analytics and problem-solving.
+At Cognizant, I’ve spent the last three years working with SQL, Python, and data tools to analyze patterns, validate reports, and troubleshoot issues—skills that align well with what you’re looking for. My experience includes writing complex SQL queries, automating data workflows, and building predictive models, like my customer churn project. I’ve also worked in small teams, which matches your collaborative environment.
+I’d welcome the chance to bring this experience to your team. Looking forward to the opportunity to discuss how I can help. Best regards, Rohit Jaiswal</t>
+  </si>
+  <si>
+    <t>Data Analyst-SQL+Power BI+Alteryx-Australian shift</t>
+  </si>
+  <si>
+    <t>PwC Service Delivery Center</t>
+  </si>
+  <si>
+    <t>https://www.naukri.com/job-listings-data-analyst-sql-power-bi-alteryx-australian-shift-pwc-service-delivery-center-kolkata-hyderabad-bengaluru-5-to-9-years-100426000179</t>
+  </si>
+  <si>
+    <t>Results-driven Data Analyst with 3+ years of experience using SQL, Python, and Power BI to extract insights and support data-driven decisions. Proficient in analyzing data, automating reporting, and troubleshooting issues using SQL, Excel, and cloud platforms. Seeking to leverage my analytics skills in a Data Analyst role supporting Australian business hours.</t>
   </si>
   <si>
     <t>Dear Hiring Team,
-I’m excited to apply for the Data Analyst role at Qualitest because I enjoy solving real-world problems with data—especially using tools like SQL and Python. Your focus on testing and analytics feels like a great fit for my background in data-driven decision-making.
-At Cognizant, I’ve spent the last three years analyzing data with SQL (MySQL/PostgreSQL) and Python to uncover trends, debug issues, and automate reporting. My experience spans writing queries, cleaning datasets with Pandas, and building predictive models—skills that align well with what you’re looking for in Google Sheets, SQL, and Linux/Unix. I’ve also worked in small teams, so I’m comfortable collaborating while owning my work independently.
-I’d love the chance to bring this experience to your team. Looking forward to the opportunity to discuss how I can contribute. Thanks for your time!</t>
-  </si>
-  <si>
-    <t>Reporting - Data Analyst</t>
-  </si>
-  <si>
-    <t>Unisys</t>
-  </si>
-  <si>
-    <t>https://in.linkedin.com/jobs/view/reporting-data-analyst-at-unisys-4408269083?position=40&amp;pageNum=0&amp;refId=tI%2FAq8zu1%2BQJFxa8XMqtSQ%3D%3D&amp;trackingId=6cSd3k6pxhZc4ElxjG5K3w%3D%3D</t>
-  </si>
-  <si>
-    <t>Detail-oriented Data Analyst with 3+ years of experience using Python, SQL, and analytics tools to generate actionable reports and insights. Skilled in extracting and validating data from MySQL and PostgreSQL, automating processes with Pandas, and identifying trends from error logs and metrics. Proficient in Azure AZ-900 and Excel, with a strong foundation in data-driven problem-solving.</t>
+I’m excited to apply for the Data Analyst role at PwC’s Service Delivery Center. The opportunity to work with SQL, Power BI, and Alteryx on real-world analytics projects—especially in an Australian shift—is a great fit for my skills and career goals.
+At Cognizant, I’ve spent over three years analyzing data with SQL and Python, building reports, and solving problems using MySQL and PostgreSQL. My work on detecting metric spikes and automating reporting aligns well with your needs, and I’ve also handled end-to-end projects like churn prediction and pension management systems. While I haven’t used Alteryx yet, my experience with Pandas and SQL gives me a strong foundation to quickly learn it.
+I’d love to bring my analytical mindset and hands-on experience to your team. Looking forward to the chance to contribute and grow at PwC.</t>
+  </si>
+  <si>
+    <t>Pico Xpress</t>
+  </si>
+  <si>
+    <t>https://www.naukri.com/job-listings-data-analyst-pico-xpress-bengaluru-3-to-5-years-300426910937</t>
+  </si>
+  <si>
+    <t>Results-driven Data Analyst with 3+ years of experience using SQL, Python, and analytics tools to uncover insights from data. Skilled in writing complex SQL queries, building reports, and applying Python (Pandas, NumPy) for data cleaning and analysis. Strong problem-solver with a track record of improving processes and delivering actionable results.</t>
   </si>
   <si>
     <t>Dear Hiring Team,
-I’m excited to apply for the Reporting Data Analyst role at Unisys because I admire how the company leverages data to drive smart business decisions. With my background in analytics and reporting, I’d love to contribute to projects where data tells meaningful stories.
-At Cognizant, I’ve spent the last three years digging into data—writing SQL queries, analyzing patterns with Python, and automating reports—to help teams make better calls. Whether it’s cleaning datasets with Pandas, validating results in MySQL/PostgreSQL, or spotting bugs through logs, I enjoy turning raw data into clear insights. My projects, like predicting customer churn and detecting metric spikes, also show how I can tackle real-world reporting challenges.
-I’d welcome the chance to bring this experience to Unisys and help turn data into actionable reports. Looking forward to the opportunity to discuss how I can contribute.</t>
+I’m excited to apply for the Data Analyst role at Pico Xpress because I love turning raw data into clear insights, and I think your focus on fast, actionable analytics aligns perfectly with my skills. Bengaluru’s growing data scene makes this opportunity even more appealing—I’d love to contribute here.
+At Cognizant, I’ve spent the last three years writing SQL queries, analyzing website data with Python (Pandas, NumPy), and building automated reports—all tasks that match your job description. My projects, like churn prediction using logistic regression and SQL-based metric analysis, show I can tackle real business problems. I’m comfortable jumping into databases (MySQL, PostgreSQL) and visualizing trends, even if I haven’t used Tableau yet.
+I’d welcome the chance to discuss how I can help your team. Looking forward to your reply!</t>
+  </si>
+  <si>
+    <t>Indium Software</t>
+  </si>
+  <si>
+    <t>https://www.naukri.com/job-listings-data-analyst-indium-software-bengaluru-1-to-4-years-191225503298</t>
+  </si>
+  <si>
+    <t>Data Analyst with 3+ years of experience using SQL, Python, and data visualization to analyze trends and generate insights. Skilled in querying databases (MySQL, PostgreSQL), cleaning data with Pandas, and building predictive models with Scikit-learn. Proven ability to automate reporting, troubleshoot issues, and collaborate in small teams.</t>
+  </si>
+  <si>
+    <t>Dear Indium Software Team,
+I’m excited to apply for the Data Analyst role at Indium Software because I admire your work in data-driven solutions, and I’m eager to bring my analytical skills to a team that values innovation. With my background in Python, SQL, and data visualization, I’m confident I can contribute meaningfully to your projects.
+At Cognizant, I’ve spent over three years analyzing data to uncover insights, writing complex SQL queries, and automating reporting—skills that align closely with what you’re looking for. My experience with tools like Pandas, NumPy, and MySQL, along with hands-on projects like customer churn prediction and operations analytics, has prepared me to tackle real-world data challenges. I thrive in collaborative environments and love turning raw data into actionable findings.
+I’d welcome the opportunity to discuss how my skills can support Indium Software’s goals. Looking forward to connecting soon—thank you for your time!</t>
+  </si>
+  <si>
+    <t>Aventra Group</t>
+  </si>
+  <si>
+    <t>https://www.naukri.com/job-listings-data-analyst-aventra-group-coimbatore-bengaluru-3-to-8-years-280426008039</t>
+  </si>
+  <si>
+    <t>Data Analyst with 3+ years of experience using SQL, Python, and data visualization tools to analyze trends and generate insights. Proficient in MySQL, PostgreSQL, and reporting, with hands-on experience in identifying patterns and automating data workflows. Skilled in Tableau-ready data preparation and delivering actionable findings from complex datasets.</t>
+  </si>
+  <si>
+    <t>Dear Hiring Team,
+I’m excited to apply for the Data Analyst role at Aventra Group because I admire how the company leverages data to drive smart business decisions. With my background in data analysis and passion for turning raw data into actionable insights, I’d love to contribute to your team.
+At Cognizant, I’ve spent over three years analyzing data using SQL, Python, and tools like Pandas and PostgreSQL—skills that align closely with your requirements. I’ve written complex SQL queries for reporting, validated large datasets, and identified patterns in website metrics, much like the work described in the job posting. My projects, like predicting customer churn and automating reporting with Python, also demonstrate hands-on experience with data visualization and analytics.
+I’d welcome the chance to bring this experience to Aventra Group. Looking forward to the opportunity to discuss how I can add value to your team.</t>
+  </si>
+  <si>
+    <t>Discover Dollar Technologies</t>
+  </si>
+  <si>
+    <t>https://www.naukri.com/job-listings-data-analyst-discover-dollar-technologies-pvt-ltd-bengaluru-1-to-3-years-101125503169</t>
+  </si>
+  <si>
+    <t>Results-driven Data Analyst with 3+ years of experience using Python, SQL, and data visualization tools to extract insights and improve business decisions. Strong analytical and problem-solving skills, with a track record of automating reports, identifying trends, and collaborating in small teams. Committed to delivering accurate, actionable data to support organizational goals with excellent time management and communication.</t>
+  </si>
+  <si>
+    <t>Dear Discover Dollar Technologies team,
+I’m excited to apply for the Data Analyst role because I admire how your company uses data to solve real business problems. With my background in analytics and problem-solving, I’d love to contribute to your team and grow alongside innovative projects like yours.
+At Cognizant, I’ve spent the last three years analyzing data with Python, SQL, and tools like Pandas and NumPy to uncover patterns, generate reports, and troubleshoot issues. My work on the OUP India website involved writing complex SQL queries, validating data, and collaborating closely with small teams—skills that align well with your requirements. I’ve also built projects like a customer churn prediction model and automated reporting systems, which demonstrate my ability to turn raw data into actionable insights.
+I’d welcome the chance to bring this experience to your team and help drive impactful results. Looking forward to the possibility of discussing how I can contribute.</t>
+  </si>
+  <si>
+    <t>The Art Of Living Human Resources</t>
+  </si>
+  <si>
+    <t>https://www.naukri.com/job-listings-data-analyst-the-art-of-living-human-resource-bengaluru-2-to-4-years-230426504671</t>
+  </si>
+  <si>
+    <t>Experienced Data Analyst with 3+ years of hands-on experience using Python, SQL, and data visualization tools to analyze trends and generate reports. Skilled in MySQL, PostgreSQL, Pandas, and Excel to extract insights and automate reporting for business decisions. Proven ability to clean, process, and visualize data to support data-driven solutions.</t>
+  </si>
+  <si>
+    <t>**Dear Hiring Team,**
+I’ve always admired The Art of Living’s work in blending data with meaningful impact, and I’d love to bring my analytical skills to your team as a Data Analyst. This role feels like a great fit for my experience in turning raw data into clear, actionable insights.
+At Cognizant, I’ve spent over three years working with SQL, Python, and visualization tools to analyze patterns, generate reports, and troubleshoot data issues—exactly the kind of work your job description highlights. Whether it was writing complex SQL queries for reporting, automating data workflows with Pandas, or building dashboards to track metrics, I’ve focused on making data easy to understand and useful for decision-making. My projects, like customer churn prediction and operations analytics, also reflect this same approach.
+I’d love to discuss how my skills could support your team. Looking forward to the opportunity!</t>
   </si>
 </sst>
 </file>
@@ -1130,13 +1181,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="4"/>
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="6" max="6" width="14.2727272727273" customWidth="1"/>
     <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="255.636363636364" customWidth="1"/>
+    <col min="8" max="8" width="60" customWidth="1"/>
     <col min="9" max="9" width="80" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="18" customWidth="1"/>
@@ -1194,7 +1246,7 @@
         <v>15</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
         <v>16</v>
@@ -1202,7 +1254,7 @@
       <c r="F2" t="s">
         <v>17</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H2" t="s">
@@ -1226,16 +1278,16 @@
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
         <v>24</v>
-      </c>
-      <c r="B3" t="s">
-        <v>25</v>
       </c>
       <c r="C3" t="s">
         <v>15</v>
       </c>
       <c r="D3">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E3" t="s">
         <v>16</v>
@@ -1243,20 +1295,20 @@
       <c r="F3" t="s">
         <v>17</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" t="s">
         <v>26</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>27</v>
       </c>
-      <c r="I3" t="s">
-        <v>28</v>
-      </c>
       <c r="J3" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="K3" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="L3" t="s">
         <v>23</v>
@@ -1267,16 +1319,16 @@
     </row>
     <row r="4" spans="1:13">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
         <v>15</v>
       </c>
       <c r="D4">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E4" t="s">
         <v>16</v>
@@ -1284,14 +1336,14 @@
       <c r="F4" t="s">
         <v>17</v>
       </c>
-      <c r="G4" t="s">
-        <v>33</v>
+      <c r="G4" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="H4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="I4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="J4" t="s">
         <v>21</v>
@@ -1308,16 +1360,16 @@
     </row>
     <row r="5" spans="1:13">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
         <v>15</v>
       </c>
       <c r="D5">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E5" t="s">
         <v>16</v>
@@ -1326,13 +1378,13 @@
         <v>17</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="H5" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="I5" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="J5" t="s">
         <v>21</v>
@@ -1347,9 +1399,180 @@
         <v>17</v>
       </c>
     </row>
+    <row r="6" spans="1:13">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6">
+        <v>7</v>
+      </c>
+      <c r="E6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" t="s">
+        <v>40</v>
+      </c>
+      <c r="J6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L6" t="s">
+        <v>23</v>
+      </c>
+      <c r="M6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7">
+        <v>7</v>
+      </c>
+      <c r="E7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" t="s">
+        <v>43</v>
+      </c>
+      <c r="I7" t="s">
+        <v>44</v>
+      </c>
+      <c r="J7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" t="s">
+        <v>47</v>
+      </c>
+      <c r="I8" t="s">
+        <v>48</v>
+      </c>
+      <c r="J8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K8" t="s">
+        <v>22</v>
+      </c>
+      <c r="L8" t="s">
+        <v>23</v>
+      </c>
+      <c r="M8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9">
+        <v>7</v>
+      </c>
+      <c r="E9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H9" t="s">
+        <v>51</v>
+      </c>
+      <c r="I9" t="s">
+        <v>52</v>
+      </c>
+      <c r="J9" t="s">
+        <v>21</v>
+      </c>
+      <c r="K9" t="s">
+        <v>22</v>
+      </c>
+      <c r="L9" t="s">
+        <v>23</v>
+      </c>
+      <c r="M9" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G5" r:id="rId1" display="https://in.linkedin.com/jobs/view/reporting-data-analyst-at-unisys-4408269083?position=40&amp;pageNum=0&amp;refId=tI%2FAq8zu1%2BQJFxa8XMqtSQ%3D%3D&amp;trackingId=6cSd3k6pxhZc4ElxjG5K3w%3D%3D"/>
+    <hyperlink ref="G2" r:id="rId1" display="https://www.naukri.com/job-listings-data-analyst-virtuoso-staffing-solutions-bengaluru-2-to-6-years-241225022830"/>
+    <hyperlink ref="G3" r:id="rId2" display="https://www.naukri.com/job-listings-data-analyst-gokaldas-exports-ltd-bangalore-bengaluru-2-to-4-years-080426933843"/>
+    <hyperlink ref="G4" r:id="rId3" display="https://www.naukri.com/job-listings-data-analyst-sql-power-bi-alteryx-australian-shift-pwc-service-delivery-center-kolkata-hyderabad-bengaluru-5-to-9-years-100426000179"/>
+    <hyperlink ref="G5" r:id="rId4" display="https://www.naukri.com/job-listings-data-analyst-pico-xpress-bengaluru-3-to-5-years-300426910937"/>
+    <hyperlink ref="G6" r:id="rId5" display="https://www.naukri.com/job-listings-data-analyst-indium-software-bengaluru-1-to-4-years-191225503298"/>
+    <hyperlink ref="G7" r:id="rId6" display="https://www.naukri.com/job-listings-data-analyst-aventra-group-coimbatore-bengaluru-3-to-8-years-280426008039"/>
+    <hyperlink ref="G8" r:id="rId7" display="https://www.naukri.com/job-listings-data-analyst-discover-dollar-technologies-pvt-ltd-bengaluru-1-to-3-years-101125503169"/>
+    <hyperlink ref="G9" r:id="rId8" display="https://www.naukri.com/job-listings-data-analyst-the-art-of-living-human-resource-bengaluru-2-to-4-years-230426504671"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -1359,14 +1582,8 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="3"/>
-  <cols>
-    <col min="6" max="6" width="14.2727272727273" customWidth="1"/>
-    <col min="7" max="7" width="218.181818181818" customWidth="1"/>
-    <col min="8" max="9" width="255.636363636364" customWidth="1"/>
-    <col min="10" max="10" width="7.72727272727273" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
@@ -1420,7 +1637,7 @@
         <v>15</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
         <v>16</v>
@@ -1452,16 +1669,16 @@
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="C3" t="s">
         <v>15</v>
       </c>
       <c r="D3">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E3" t="s">
         <v>16</v>
@@ -1470,13 +1687,13 @@
         <v>17</v>
       </c>
       <c r="G3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="H3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="I3" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="J3" t="s">
         <v>21</v>
@@ -1493,16 +1710,16 @@
     </row>
     <row r="4" spans="1:13">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
         <v>15</v>
       </c>
       <c r="D4">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E4" t="s">
         <v>16</v>
@@ -1511,13 +1728,13 @@
         <v>17</v>
       </c>
       <c r="G4" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="H4" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="I4" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="J4" t="s">
         <v>21</v>
@@ -1529,6 +1746,211 @@
         <v>23</v>
       </c>
       <c r="M4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5">
+        <v>9</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K5" t="s">
+        <v>22</v>
+      </c>
+      <c r="L5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6">
+        <v>7</v>
+      </c>
+      <c r="E6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" t="s">
+        <v>40</v>
+      </c>
+      <c r="J6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L6" t="s">
+        <v>23</v>
+      </c>
+      <c r="M6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7">
+        <v>7</v>
+      </c>
+      <c r="E7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" t="s">
+        <v>43</v>
+      </c>
+      <c r="I7" t="s">
+        <v>44</v>
+      </c>
+      <c r="J7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" t="s">
+        <v>47</v>
+      </c>
+      <c r="I8" t="s">
+        <v>48</v>
+      </c>
+      <c r="J8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K8" t="s">
+        <v>22</v>
+      </c>
+      <c r="L8" t="s">
+        <v>23</v>
+      </c>
+      <c r="M8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9">
+        <v>7</v>
+      </c>
+      <c r="E9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" t="s">
+        <v>50</v>
+      </c>
+      <c r="H9" t="s">
+        <v>51</v>
+      </c>
+      <c r="I9" t="s">
+        <v>52</v>
+      </c>
+      <c r="J9" t="s">
+        <v>21</v>
+      </c>
+      <c r="K9" t="s">
+        <v>22</v>
+      </c>
+      <c r="L9" t="s">
+        <v>23</v>
+      </c>
+      <c r="M9" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1541,7 +1963,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:13">
@@ -1585,6 +2007,334 @@
         <v>12</v>
       </c>
     </row>
+    <row r="2" spans="1:13">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5">
+        <v>9</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K5" t="s">
+        <v>22</v>
+      </c>
+      <c r="L5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6">
+        <v>7</v>
+      </c>
+      <c r="E6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" t="s">
+        <v>40</v>
+      </c>
+      <c r="J6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L6" t="s">
+        <v>23</v>
+      </c>
+      <c r="M6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7">
+        <v>7</v>
+      </c>
+      <c r="E7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" t="s">
+        <v>43</v>
+      </c>
+      <c r="I7" t="s">
+        <v>44</v>
+      </c>
+      <c r="J7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" t="s">
+        <v>47</v>
+      </c>
+      <c r="I8" t="s">
+        <v>48</v>
+      </c>
+      <c r="J8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K8" t="s">
+        <v>22</v>
+      </c>
+      <c r="L8" t="s">
+        <v>23</v>
+      </c>
+      <c r="M8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9">
+        <v>7</v>
+      </c>
+      <c r="E9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" t="s">
+        <v>50</v>
+      </c>
+      <c r="H9" t="s">
+        <v>51</v>
+      </c>
+      <c r="I9" t="s">
+        <v>52</v>
+      </c>
+      <c r="J9" t="s">
+        <v>21</v>
+      </c>
+      <c r="K9" t="s">
+        <v>22</v>
+      </c>
+      <c r="L9" t="s">
+        <v>23</v>
+      </c>
+      <c r="M9" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>